<commit_message>
Removed duplicatelines from Config.properties
</commit_message>
<xml_diff>
--- a/ServiceWA/ExtentUtilities/File/Extent.xlsx
+++ b/ServiceWA/ExtentUtilities/File/Extent.xlsx
@@ -14,12 +14,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>TestcaseID-Stability_TC_01_Mobile validate Linkable service FishCatchWA</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+  <si>
+    <t>TestcaseID-Stability_TC_02_Mobile Validation of login</t>
   </si>
   <si>
     <t>ServiceWA Application</t>
+  </si>
+  <si>
+    <t>GotIt Button is not visible</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/15-14-55/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Done Button is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/15-14-57/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Continue Button is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/15-14-59/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Settings Icon is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/15-15-34/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>LoginToServiceWA Button is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/15-15-36/PassedStep.jpg</t>
   </si>
 </sst>
 </file>
@@ -351,15 +384,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
worked on the login scenario and add test steps  ServiceWA_Login.robot, SignInScreen.robot
</commit_message>
<xml_diff>
--- a/ServiceWA/ExtentUtilities/File/Extent.xlsx
+++ b/ServiceWA/ExtentUtilities/File/Extent.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
   <si>
     <t>TestcaseID-Stability_TC_02_Mobile Validation of login</t>
   </si>
@@ -28,31 +28,52 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/16-Mar-2026/15-14-55/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-15-59/PassedStep.jpg</t>
   </si>
   <si>
     <t>Done Button is not visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/16-Mar-2026/15-14-57/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-01/PassedStep.jpg</t>
   </si>
   <si>
     <t>Continue Button is not visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/16-Mar-2026/15-14-59/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-03/PassedStep.jpg</t>
   </si>
   <si>
     <t>Settings Icon is not visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/16-Mar-2026/15-15-34/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-06/PassedStep.jpg</t>
   </si>
   <si>
     <t>LoginToServiceWA Button is not visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/16-Mar-2026/15-15-36/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-14/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>IAgree Button is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-22/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Next Button is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-24/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>ReadyToBegin Button is not visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-27/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/16-Mar-2026/21-16-29/PassedStep.jpg</t>
   </si>
 </sst>
 </file>
@@ -384,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -450,6 +471,50 @@
         <v>12</v>
       </c>
     </row>
+    <row r="7" spans="1:4">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Modified ServiceWA_Login.robot and Added some method in AppiumCommon.robot
</commit_message>
<xml_diff>
--- a/ServiceWA/ExtentUtilities/File/Extent.xlsx
+++ b/ServiceWA/ExtentUtilities/File/Extent.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
   <si>
     <t>TestcaseID-Stability_TC_02_Mobile Validation of login</t>
   </si>
@@ -28,55 +28,55 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-57-44/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-02-46/PassedStep.jpg</t>
   </si>
   <si>
     <t>Done Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-57-46/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-02-48/PassedStep.jpg</t>
   </si>
   <si>
     <t>Continue Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-57-50/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-02-53/PassedStep.jpg</t>
   </si>
   <si>
     <t>Settings Icon is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-57-59/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-02/PassedStep.jpg</t>
   </si>
   <si>
     <t>LoginToServiceWA Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-58-02/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-05/PassedStep.jpg</t>
   </si>
   <si>
     <t>IAgree Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-58-10/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-13/PassedStep.jpg</t>
   </si>
   <si>
     <t>Next Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-58-13/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-16/PassedStep.jpg</t>
   </si>
   <si>
     <t>ReadyToBegin Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-58-15/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-19/PassedStep.jpg</t>
   </si>
   <si>
     <t>ContinueWithDigitalID Link is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-58-18/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-22/PassedStep.jpg</t>
   </si>
   <si>
     <t>SelectMyID Button is not visible</t>
@@ -85,46 +85,52 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-58-59/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-04-02/PassedStep.jpg</t>
   </si>
   <si>
     <t>SGetCode Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/09-59-16/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-04-18/PassedStep.jpg</t>
   </si>
   <si>
     <t>Consent Button is not visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/10-00-00/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-03/PassedStep.jpg</t>
   </si>
   <si>
     <t>FinalConsent Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/10-00-10/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/10-00-14/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-12/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-16/PassedStep.jpg</t>
   </si>
   <si>
     <t>SkipForNow Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/10-00-17/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-19/PassedStep.jpg</t>
   </si>
   <si>
     <t>YesSkip Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/10-00-19/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-22/PassedStep.jpg</t>
   </si>
   <si>
     <t>LogOut Button is visible</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/10-00-22/PassedStep.jpg</t>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-25/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Close Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-28/PassedStep.jpg</t>
   </si>
 </sst>
 </file>
@@ -456,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -654,6 +660,17 @@
         <v>36</v>
       </c>
     </row>
+    <row r="19" spans="2:4">
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Login testcase compleeted and updated
</commit_message>
<xml_diff>
--- a/ServiceWA/ExtentUtilities/File/Extent.xlsx
+++ b/ServiceWA/ExtentUtilities/File/Extent.xlsx
@@ -14,123 +14,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
-  <si>
-    <t>TestcaseID-Stability_TC_02_Mobile Validation of login</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Login001-Stability_TC_01_Mobile Before login Steps</t>
   </si>
   <si>
     <t>ServiceWA Application</t>
   </si>
   <si>
-    <t>GotIt Button is visible</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-02-46/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>Done Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-02-48/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>Continue Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-02-53/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>Settings Icon is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-02/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>LoginToServiceWA Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-05/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>IAgree Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-13/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>Next Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-16/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>ReadyToBegin Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-19/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>ContinueWithDigitalID Link is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-03-22/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>SelectMyID Button is not visible</t>
+    <t>Exception Occurred; Element didn't appear. //android.widget.Button[@content-desc="Got it"]</t>
   </si>
   <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-04-02/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>SGetCode Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-04-18/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>Consent Button is not visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-03/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>FinalConsent Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-12/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-16/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>SkipForNow Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-19/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>YesSkip Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-22/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>LogOut Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-25/PassedStep.jpg</t>
-  </si>
-  <si>
-    <t>Close Button is visible</t>
-  </si>
-  <si>
-    <t>./Screenshots/TestcaseID/20-Mar-2026/12-05-28/PassedStep.jpg</t>
+    <t>./Screenshots/Login001/20-Mar-2026/15-25-23/PassedStep.jpg</t>
   </si>
 </sst>
 </file>
@@ -462,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -484,193 +382,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
-        <v>3</v>
-      </c>
-      <c r="D12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="B14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="B15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="B16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4">
-      <c r="B17" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4">
-      <c r="B18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4">
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>3</v>
-      </c>
-      <c r="D19" t="s">
-        <v>38</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
FuelWatch method developed it is working fine in IOS
</commit_message>
<xml_diff>
--- a/ServiceWA/ExtentUtilities/File/Extent.xlsx
+++ b/ServiceWA/ExtentUtilities/File/Extent.xlsx
@@ -14,21 +14,81 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>Login001-Stability_TC_01_Mobile Before login Steps</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
+  <si>
+    <t>Login001-Stability_TC_01_Mobile validate_ Linkable service FuelWatch</t>
   </si>
   <si>
     <t>ServiceWA Application</t>
   </si>
   <si>
-    <t>Exception Occurred; Element didn't appear. //android.widget.Button[@content-desc="Got it"]</t>
+    <t>GotIt Button is visible</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-05-39/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Done Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-05-41/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Continue Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-05-47/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>LinkableServices Button is not visible</t>
   </si>
   <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>./Screenshots/Login001/20-Mar-2026/15-25-23/PassedStep.jpg</t>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-24/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>FuelWatch Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-27/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Next Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-30/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>IAgree Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-38/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>AcceptLocationService Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-43/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>FuelWatchBackToServiceWA Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-45/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-49/PassedStep.jpg</t>
+  </si>
+  <si>
+    <t>Linked Button is visible</t>
+  </si>
+  <si>
+    <t>./Screenshots/Login001/24-Mar-2026/00-06-52/PassedStep.jpg</t>
   </si>
 </sst>
 </file>
@@ -360,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -382,6 +442,116 @@
         <v>4</v>
       </c>
     </row>
+    <row r="3" spans="1:4">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>